<commit_message>
feat: Enhance Excel processing and analysis
- Added RTL file path and conditions to the JSON structure in `fill_define_excel_if_needed`.
- Improved logging in `fill_define.py` for better debugging of signal assignments.
- Introduced `analyze_excel.py` to analyze the structure of the Excel file and check for 'Signal Assignments'.
- Created `test_find_header.py` to test the `find_signal_assignments_header` function against the Excel data.
- Updated binary files for the Excel and compiled Python files.
</commit_message>
<xml_diff>
--- a/out/sessions/sfr_cap-20251014_191534/sfr_cap.xlsx
+++ b/out/sessions/sfr_cap-20251014_191534/sfr_cap.xlsx
@@ -5827,7 +5827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:V36"/>
+  <dimension ref="B3:V36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -5854,8 +5854,6 @@
     <col width="3.125" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="19.5" customHeight="1">
       <c r="B3" s="105" t="inlineStr">
         <is>
@@ -6181,7 +6179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:M38"/>
+  <dimension ref="B3:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -6192,8 +6190,6 @@
     <col width="4" customWidth="1" style="43" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3">
       <c r="I3" t="n"/>
     </row>
@@ -6376,7 +6372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AQ139"/>
+  <dimension ref="B2:AQ71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -6388,7 +6384,6 @@
     <col width="3.125" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="I2" t="inlineStr">
         <is>
@@ -6417,8 +6412,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8" ht="21" customHeight="1">
       <c r="B8" s="72" t="n"/>
       <c r="C8" s="38" t="inlineStr">
@@ -6918,8 +6911,6 @@
       <c r="F40" s="7" t="n"/>
     </row>
     <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
     <row r="44" ht="20.25" customHeight="1">
       <c r="I44" s="113" t="inlineStr">
         <is>
@@ -6981,74 +6972,6 @@
     <row r="69"/>
     <row r="70"/>
     <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="I22:S41"/>
@@ -7075,7 +6998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Q36"/>
+  <dimension ref="B3:Q36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -7086,8 +7009,6 @@
     <col width="3.125" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="19.5" customHeight="1">
       <c r="C3" s="204" t="inlineStr">
         <is>
@@ -7248,7 +7169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:T18"/>
+  <dimension ref="C2:T18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -7261,7 +7182,6 @@
     <col width="3.125" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="C2" t="inlineStr">
         <is>
@@ -7440,7 +7360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:V36"/>
+  <dimension ref="B3:V36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" min="1" max="1"/>
@@ -7467,8 +7387,6 @@
     <col width="3.125" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="19.5" customHeight="1">
       <c r="B3" s="105" t="inlineStr">
         <is>
@@ -9591,11 +9509,6 @@
       <c r="Q45" s="215" t="n"/>
       <c r="R45" s="216" t="n"/>
     </row>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="V26:V27"/>

</xml_diff>